<commit_message>
Updated README and OCLTLoc case studies
</commit_message>
<xml_diff>
--- a/LiTeLLab/Scalability.xlsx
+++ b/LiTeLLab/Scalability.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pourhashem\Dropbox\mazust\Research\OLTL-Optimization LTL\litellabGit\LiTeLLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA93B788-80EA-4CDC-90D2-83FC095FF6AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAF2494E-95F1-495E-9835-CE4B107C53A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AL" sheetId="2" r:id="rId1"/>
@@ -1043,10 +1043,40 @@
     <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1055,175 +1085,145 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2556,12 +2556,12 @@
       <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="17" t="s">
+      <c r="G1" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -2590,7 +2590,7 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="16">
+      <c r="A3" s="29">
         <v>19</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -2602,7 +2602,7 @@
       <c r="D3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="28" t="s">
         <v>37</v>
       </c>
       <c r="F3" s="4">
@@ -2622,7 +2622,7 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="16"/>
+      <c r="A4" s="29"/>
       <c r="B4" s="1" t="s">
         <v>6</v>
       </c>
@@ -2632,7 +2632,7 @@
       <c r="D4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="18"/>
+      <c r="E4" s="28"/>
       <c r="F4" s="4">
         <v>16</v>
       </c>
@@ -2650,7 +2650,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="16"/>
+      <c r="A5" s="29"/>
       <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
@@ -2660,7 +2660,7 @@
       <c r="D5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="18"/>
+      <c r="E5" s="28"/>
       <c r="F5" s="4">
         <v>17</v>
       </c>
@@ -2678,7 +2678,7 @@
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="16"/>
+      <c r="A6" s="29"/>
       <c r="B6" s="1" t="s">
         <v>8</v>
       </c>
@@ -2688,7 +2688,7 @@
       <c r="D6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="18"/>
+      <c r="E6" s="28"/>
       <c r="F6" s="4">
         <v>18</v>
       </c>
@@ -2706,7 +2706,7 @@
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="16">
+      <c r="A7" s="29">
         <v>20</v>
       </c>
       <c r="B7" s="1" t="s">
@@ -2718,7 +2718,7 @@
       <c r="D7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="18"/>
+      <c r="E7" s="28"/>
       <c r="F7" s="4">
         <v>19</v>
       </c>
@@ -2736,7 +2736,7 @@
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="16"/>
+      <c r="A8" s="29"/>
       <c r="B8" s="1" t="s">
         <v>10</v>
       </c>
@@ -2746,7 +2746,7 @@
       <c r="D8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="18"/>
+      <c r="E8" s="28"/>
       <c r="F8" s="4">
         <v>20</v>
       </c>
@@ -2764,7 +2764,7 @@
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="16"/>
+      <c r="A9" s="29"/>
       <c r="B9" s="1" t="s">
         <v>11</v>
       </c>
@@ -2774,7 +2774,7 @@
       <c r="D9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="18"/>
+      <c r="E9" s="28"/>
       <c r="F9" s="4">
         <v>21</v>
       </c>
@@ -2792,7 +2792,7 @@
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="16"/>
+      <c r="A10" s="29"/>
       <c r="B10" s="1" t="s">
         <v>12</v>
       </c>
@@ -2802,7 +2802,7 @@
       <c r="D10" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E10" s="18"/>
+      <c r="E10" s="28"/>
       <c r="F10" s="4">
         <v>22</v>
       </c>
@@ -2820,7 +2820,7 @@
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="16">
+      <c r="A11" s="29">
         <v>21</v>
       </c>
       <c r="B11" s="1" t="s">
@@ -2832,7 +2832,7 @@
       <c r="D11" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E11" s="18"/>
+      <c r="E11" s="28"/>
       <c r="F11" s="4">
         <v>23</v>
       </c>
@@ -2850,7 +2850,7 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="16"/>
+      <c r="A12" s="29"/>
       <c r="B12" s="1" t="s">
         <v>14</v>
       </c>
@@ -2860,7 +2860,7 @@
       <c r="D12" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E12" s="18"/>
+      <c r="E12" s="28"/>
       <c r="F12" s="4">
         <v>24</v>
       </c>
@@ -2878,7 +2878,7 @@
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="16"/>
+      <c r="A13" s="29"/>
       <c r="B13" s="1" t="s">
         <v>15</v>
       </c>
@@ -2888,7 +2888,7 @@
       <c r="D13" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E13" s="18"/>
+      <c r="E13" s="28"/>
       <c r="F13" s="4">
         <v>25</v>
       </c>
@@ -2906,7 +2906,7 @@
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="16"/>
+      <c r="A14" s="29"/>
       <c r="B14" s="1" t="s">
         <v>16</v>
       </c>
@@ -2918,7 +2918,7 @@
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="16">
+      <c r="A15" s="29">
         <v>22</v>
       </c>
       <c r="B15" s="1" t="s">
@@ -2932,7 +2932,7 @@
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="16"/>
+      <c r="A16" s="29"/>
       <c r="B16" s="1" t="s">
         <v>18</v>
       </c>
@@ -2956,7 +2956,7 @@
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="16"/>
+      <c r="A17" s="29"/>
       <c r="B17" s="1" t="s">
         <v>19</v>
       </c>
@@ -2968,7 +2968,7 @@
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="16"/>
+      <c r="A18" s="29"/>
       <c r="B18" s="1" t="s">
         <v>20</v>
       </c>
@@ -2980,7 +2980,7 @@
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="16">
+      <c r="A19" s="29">
         <v>23</v>
       </c>
       <c r="B19" s="1" t="s">
@@ -2994,7 +2994,7 @@
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="16"/>
+      <c r="A20" s="29"/>
       <c r="B20" s="1" t="s">
         <v>22</v>
       </c>
@@ -3006,7 +3006,7 @@
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="16"/>
+      <c r="A21" s="29"/>
       <c r="B21" s="1" t="s">
         <v>23</v>
       </c>
@@ -3018,7 +3018,7 @@
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="16"/>
+      <c r="A22" s="29"/>
       <c r="B22" s="1" t="s">
         <v>24</v>
       </c>
@@ -3030,7 +3030,7 @@
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="16">
+      <c r="A23" s="29">
         <v>24</v>
       </c>
       <c r="B23" s="1" t="s">
@@ -3044,7 +3044,7 @@
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" s="16"/>
+      <c r="A24" s="29"/>
       <c r="B24" s="1" t="s">
         <v>26</v>
       </c>
@@ -3056,7 +3056,7 @@
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" s="16"/>
+      <c r="A25" s="29"/>
       <c r="B25" s="1" t="s">
         <v>27</v>
       </c>
@@ -3068,7 +3068,7 @@
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26" s="16"/>
+      <c r="A26" s="29"/>
       <c r="B26" s="1" t="s">
         <v>28</v>
       </c>
@@ -3080,7 +3080,7 @@
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A27" s="16">
+      <c r="A27" s="29">
         <v>25</v>
       </c>
       <c r="B27" s="1" t="s">
@@ -3094,7 +3094,7 @@
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A28" s="16"/>
+      <c r="A28" s="29"/>
       <c r="B28" s="1" t="s">
         <v>30</v>
       </c>
@@ -3107,18 +3107,18 @@
       <c r="L28" s="2">
         <v>4</v>
       </c>
-      <c r="M28" s="15">
+      <c r="M28" s="26">
         <v>3</v>
       </c>
-      <c r="N28" s="15">
+      <c r="N28" s="26">
         <v>2</v>
       </c>
-      <c r="O28" s="15">
+      <c r="O28" s="26">
         <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A29" s="16"/>
+      <c r="A29" s="29"/>
       <c r="B29" s="1" t="s">
         <v>31</v>
       </c>
@@ -3131,15 +3131,15 @@
       <c r="K29" s="2">
         <v>6</v>
       </c>
-      <c r="L29" s="15">
+      <c r="L29" s="26">
         <v>5</v>
       </c>
-      <c r="M29" s="15"/>
-      <c r="N29" s="15"/>
-      <c r="O29" s="15"/>
+      <c r="M29" s="26"/>
+      <c r="N29" s="26"/>
+      <c r="O29" s="26"/>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A30" s="16"/>
+      <c r="A30" s="29"/>
       <c r="B30" s="1" t="s">
         <v>32</v>
       </c>
@@ -3152,10 +3152,10 @@
       <c r="K30" s="2">
         <v>7</v>
       </c>
-      <c r="L30" s="15"/>
-      <c r="M30" s="15"/>
-      <c r="N30" s="15"/>
-      <c r="O30" s="15"/>
+      <c r="L30" s="26"/>
+      <c r="M30" s="26"/>
+      <c r="N30" s="26"/>
+      <c r="O30" s="26"/>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="K31" s="2">
@@ -3164,36 +3164,36 @@
       <c r="L31" s="2">
         <v>10</v>
       </c>
-      <c r="M31" s="15">
+      <c r="M31" s="26">
         <v>9</v>
       </c>
-      <c r="N31" s="15">
+      <c r="N31" s="26">
         <v>8</v>
       </c>
-      <c r="O31" s="15"/>
+      <c r="O31" s="26"/>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="L32" s="2">
         <v>12</v>
       </c>
-      <c r="M32" s="15"/>
-      <c r="N32" s="15"/>
-      <c r="O32" s="15"/>
+      <c r="M32" s="26"/>
+      <c r="N32" s="26"/>
+      <c r="O32" s="26"/>
     </row>
     <row r="34" spans="11:15" x14ac:dyDescent="0.25">
       <c r="K34" s="2">
         <v>17</v>
       </c>
-      <c r="L34" s="15">
+      <c r="L34" s="26">
         <v>16</v>
       </c>
-      <c r="M34" s="15">
+      <c r="M34" s="26">
         <v>15</v>
       </c>
-      <c r="N34" s="15">
+      <c r="N34" s="26">
         <v>14</v>
       </c>
-      <c r="O34" s="15">
+      <c r="O34" s="26">
         <v>13</v>
       </c>
     </row>
@@ -3201,40 +3201,35 @@
       <c r="K35" s="2">
         <v>18</v>
       </c>
-      <c r="L35" s="15"/>
-      <c r="M35" s="15"/>
-      <c r="N35" s="15"/>
-      <c r="O35" s="15"/>
+      <c r="L35" s="26"/>
+      <c r="M35" s="26"/>
+      <c r="N35" s="26"/>
+      <c r="O35" s="26"/>
     </row>
     <row r="36" spans="11:15" x14ac:dyDescent="0.25">
       <c r="K36" s="2">
         <v>21</v>
       </c>
-      <c r="L36" s="15">
+      <c r="L36" s="26">
         <v>20</v>
       </c>
-      <c r="M36" s="15">
+      <c r="M36" s="26">
         <v>19</v>
       </c>
-      <c r="N36" s="15"/>
-      <c r="O36" s="15"/>
+      <c r="N36" s="26"/>
+      <c r="O36" s="26"/>
     </row>
     <row r="37" spans="11:15" x14ac:dyDescent="0.25">
       <c r="K37" s="2">
         <v>22</v>
       </c>
-      <c r="L37" s="15"/>
-      <c r="M37" s="15"/>
-      <c r="N37" s="15"/>
-      <c r="O37" s="15"/>
+      <c r="L37" s="26"/>
+      <c r="M37" s="26"/>
+      <c r="N37" s="26"/>
+      <c r="O37" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="M36:M37"/>
-    <mergeCell ref="G1:J1"/>
-    <mergeCell ref="E3:E13"/>
-    <mergeCell ref="L34:L35"/>
-    <mergeCell ref="M34:M35"/>
     <mergeCell ref="N34:N37"/>
     <mergeCell ref="O34:O37"/>
     <mergeCell ref="A3:A6"/>
@@ -3251,6 +3246,11 @@
     <mergeCell ref="N31:N32"/>
     <mergeCell ref="A27:A30"/>
     <mergeCell ref="L36:L37"/>
+    <mergeCell ref="M36:M37"/>
+    <mergeCell ref="G1:J1"/>
+    <mergeCell ref="E3:E13"/>
+    <mergeCell ref="L34:L35"/>
+    <mergeCell ref="M34:M35"/>
   </mergeCells>
   <conditionalFormatting sqref="C1:C32 C36:C1048576">
     <cfRule type="colorScale" priority="4">
@@ -3328,7 +3328,7 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="16">
+      <c r="A3" s="29">
         <v>19</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -3339,7 +3339,7 @@
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="16"/>
+      <c r="A4" s="29"/>
       <c r="B4" s="1" t="s">
         <v>6</v>
       </c>
@@ -3348,7 +3348,7 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="16"/>
+      <c r="A5" s="29"/>
       <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
@@ -3357,7 +3357,7 @@
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="16"/>
+      <c r="A6" s="29"/>
       <c r="B6" s="1" t="s">
         <v>8</v>
       </c>
@@ -3366,7 +3366,7 @@
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="16">
+      <c r="A7" s="29">
         <v>20</v>
       </c>
       <c r="B7" s="1" t="s">
@@ -3377,7 +3377,7 @@
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="16"/>
+      <c r="A8" s="29"/>
       <c r="B8" s="1" t="s">
         <v>10</v>
       </c>
@@ -3386,7 +3386,7 @@
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="16"/>
+      <c r="A9" s="29"/>
       <c r="B9" s="1" t="s">
         <v>11</v>
       </c>
@@ -3395,7 +3395,7 @@
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="16"/>
+      <c r="A10" s="29"/>
       <c r="B10" s="1" t="s">
         <v>12</v>
       </c>
@@ -3404,7 +3404,7 @@
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="16">
+      <c r="A11" s="29">
         <v>21</v>
       </c>
       <c r="B11" s="1" t="s">
@@ -3415,7 +3415,7 @@
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="16"/>
+      <c r="A12" s="29"/>
       <c r="B12" s="1" t="s">
         <v>14</v>
       </c>
@@ -3424,7 +3424,7 @@
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="16"/>
+      <c r="A13" s="29"/>
       <c r="B13" s="1" t="s">
         <v>15</v>
       </c>
@@ -3433,7 +3433,7 @@
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="16"/>
+      <c r="A14" s="29"/>
       <c r="B14" s="1" t="s">
         <v>16</v>
       </c>
@@ -3442,7 +3442,7 @@
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="16">
+      <c r="A15" s="29">
         <v>22</v>
       </c>
       <c r="B15" s="1" t="s">
@@ -3453,7 +3453,7 @@
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="16"/>
+      <c r="A16" s="29"/>
       <c r="B16" s="1" t="s">
         <v>18</v>
       </c>
@@ -3462,7 +3462,7 @@
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" s="16"/>
+      <c r="A17" s="29"/>
       <c r="B17" s="1" t="s">
         <v>19</v>
       </c>
@@ -3471,7 +3471,7 @@
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="16"/>
+      <c r="A18" s="29"/>
       <c r="B18" s="1" t="s">
         <v>20</v>
       </c>
@@ -3480,7 +3480,7 @@
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="16">
+      <c r="A19" s="29">
         <v>23</v>
       </c>
       <c r="B19" s="1" t="s">
@@ -3494,7 +3494,7 @@
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" s="16"/>
+      <c r="A20" s="29"/>
       <c r="B20" s="1" t="s">
         <v>22</v>
       </c>
@@ -3504,18 +3504,18 @@
       <c r="G20" s="1">
         <v>4</v>
       </c>
-      <c r="H20" s="16">
+      <c r="H20" s="29">
         <v>3</v>
       </c>
-      <c r="I20" s="16">
+      <c r="I20" s="29">
         <v>2</v>
       </c>
-      <c r="J20" s="16">
+      <c r="J20" s="29">
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A21" s="16"/>
+      <c r="A21" s="29"/>
       <c r="B21" s="1" t="s">
         <v>23</v>
       </c>
@@ -3525,15 +3525,15 @@
       <c r="F21" s="1">
         <v>6</v>
       </c>
-      <c r="G21" s="16">
+      <c r="G21" s="29">
         <v>5</v>
       </c>
-      <c r="H21" s="16"/>
-      <c r="I21" s="16"/>
-      <c r="J21" s="16"/>
+      <c r="H21" s="29"/>
+      <c r="I21" s="29"/>
+      <c r="J21" s="29"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="16"/>
+      <c r="A22" s="29"/>
       <c r="B22" s="1" t="s">
         <v>24</v>
       </c>
@@ -3543,13 +3543,13 @@
       <c r="F22" s="1">
         <v>7</v>
       </c>
-      <c r="G22" s="16"/>
-      <c r="H22" s="16"/>
-      <c r="I22" s="16"/>
-      <c r="J22" s="16"/>
+      <c r="G22" s="29"/>
+      <c r="H22" s="29"/>
+      <c r="I22" s="29"/>
+      <c r="J22" s="29"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" s="16">
+      <c r="A23" s="29">
         <v>24</v>
       </c>
       <c r="B23" s="1" t="s">
@@ -3564,16 +3564,16 @@
       <c r="G23" s="1">
         <v>10</v>
       </c>
-      <c r="H23" s="16">
+      <c r="H23" s="29">
         <v>9</v>
       </c>
-      <c r="I23" s="16">
+      <c r="I23" s="29">
         <v>8</v>
       </c>
-      <c r="J23" s="16"/>
+      <c r="J23" s="29"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" s="16"/>
+      <c r="A24" s="29"/>
       <c r="B24" s="1" t="s">
         <v>26</v>
       </c>
@@ -3583,12 +3583,12 @@
       <c r="G24" s="1">
         <v>12</v>
       </c>
-      <c r="H24" s="16"/>
-      <c r="I24" s="16"/>
-      <c r="J24" s="16"/>
+      <c r="H24" s="29"/>
+      <c r="I24" s="29"/>
+      <c r="J24" s="29"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A25" s="16"/>
+      <c r="A25" s="29"/>
       <c r="B25" s="1" t="s">
         <v>27</v>
       </c>
@@ -3597,7 +3597,7 @@
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A26" s="16"/>
+      <c r="A26" s="29"/>
       <c r="B26" s="1" t="s">
         <v>28</v>
       </c>
@@ -3607,21 +3607,21 @@
       <c r="F26" s="1">
         <v>17</v>
       </c>
-      <c r="G26" s="16">
+      <c r="G26" s="29">
         <v>16</v>
       </c>
-      <c r="H26" s="16">
+      <c r="H26" s="29">
         <v>15</v>
       </c>
-      <c r="I26" s="16">
+      <c r="I26" s="29">
         <v>14</v>
       </c>
-      <c r="J26" s="16">
+      <c r="J26" s="29">
         <v>13</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A27" s="16">
+      <c r="A27" s="29">
         <v>25</v>
       </c>
       <c r="B27" s="1" t="s">
@@ -3633,13 +3633,13 @@
       <c r="F27" s="1">
         <v>18</v>
       </c>
-      <c r="G27" s="16"/>
-      <c r="H27" s="16"/>
-      <c r="I27" s="16"/>
-      <c r="J27" s="16"/>
+      <c r="G27" s="29"/>
+      <c r="H27" s="29"/>
+      <c r="I27" s="29"/>
+      <c r="J27" s="29"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" s="16"/>
+      <c r="A28" s="29"/>
       <c r="B28" s="1" t="s">
         <v>30</v>
       </c>
@@ -3649,17 +3649,17 @@
       <c r="F28" s="1">
         <v>21</v>
       </c>
-      <c r="G28" s="16">
+      <c r="G28" s="29">
         <v>20</v>
       </c>
-      <c r="H28" s="16">
+      <c r="H28" s="29">
         <v>19</v>
       </c>
-      <c r="I28" s="16"/>
-      <c r="J28" s="16"/>
+      <c r="I28" s="29"/>
+      <c r="J28" s="29"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A29" s="16"/>
+      <c r="A29" s="29"/>
       <c r="B29" s="1" t="s">
         <v>31</v>
       </c>
@@ -3669,13 +3669,13 @@
       <c r="F29" s="1">
         <v>22</v>
       </c>
-      <c r="G29" s="16"/>
-      <c r="H29" s="16"/>
-      <c r="I29" s="16"/>
-      <c r="J29" s="16"/>
+      <c r="G29" s="29"/>
+      <c r="H29" s="29"/>
+      <c r="I29" s="29"/>
+      <c r="J29" s="29"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A30" s="16"/>
+      <c r="A30" s="29"/>
       <c r="B30" s="1" t="s">
         <v>32</v>
       </c>
@@ -3685,11 +3685,6 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="A3:A6"/>
-    <mergeCell ref="A7:A10"/>
-    <mergeCell ref="A11:A14"/>
-    <mergeCell ref="A15:A18"/>
-    <mergeCell ref="A19:A22"/>
     <mergeCell ref="I23:I24"/>
     <mergeCell ref="J20:J24"/>
     <mergeCell ref="J26:J29"/>
@@ -3704,6 +3699,11 @@
     <mergeCell ref="H26:H27"/>
     <mergeCell ref="H28:H29"/>
     <mergeCell ref="A23:A26"/>
+    <mergeCell ref="A3:A6"/>
+    <mergeCell ref="A7:A10"/>
+    <mergeCell ref="A11:A14"/>
+    <mergeCell ref="A15:A18"/>
+    <mergeCell ref="A19:A22"/>
   </mergeCells>
   <conditionalFormatting sqref="C1:C32 C36:C1048576">
     <cfRule type="colorScale" priority="2">
@@ -3740,12 +3740,12 @@
   <sheetData>
     <row r="3" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="L4" s="71" t="s">
+      <c r="L4" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="M4" s="72"/>
-      <c r="N4" s="72"/>
-      <c r="O4" s="73"/>
+      <c r="M4" s="31"/>
+      <c r="N4" s="31"/>
+      <c r="O4" s="32"/>
     </row>
     <row r="5" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
@@ -3766,22 +3766,22 @@
       <c r="G5" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="I5" s="68" t="s">
+      <c r="I5" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="J5" s="69" t="s">
+      <c r="J5" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="L5" s="68" t="s">
+      <c r="L5" s="21" t="s">
         <v>72</v>
       </c>
-      <c r="M5" s="75" t="s">
+      <c r="M5" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="N5" s="75" t="s">
+      <c r="N5" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="O5" s="69" t="s">
+      <c r="O5" s="22" t="s">
         <v>75</v>
       </c>
     </row>
@@ -3806,22 +3806,22 @@
       <c r="G6" s="1">
         <v>49</v>
       </c>
-      <c r="I6" s="66">
+      <c r="I6" s="19">
         <v>4</v>
       </c>
-      <c r="J6" s="67">
+      <c r="J6" s="20">
         <v>9</v>
       </c>
-      <c r="L6" s="66">
+      <c r="L6" s="19">
         <v>49</v>
       </c>
-      <c r="M6" s="74">
+      <c r="M6" s="24">
         <v>70</v>
       </c>
-      <c r="N6" s="74">
+      <c r="N6" s="24">
         <v>77</v>
       </c>
-      <c r="O6" s="67">
+      <c r="O6" s="20">
         <v>60</v>
       </c>
     </row>
@@ -3846,13 +3846,13 @@
       <c r="G7" s="1">
         <v>70</v>
       </c>
-      <c r="I7" s="62">
+      <c r="I7" s="15">
         <v>5</v>
       </c>
-      <c r="J7" s="63">
+      <c r="J7" s="16">
         <v>12</v>
       </c>
-      <c r="L7" s="62">
+      <c r="L7" s="15">
         <v>132</v>
       </c>
       <c r="M7" s="2">
@@ -3861,7 +3861,7 @@
       <c r="N7" s="2">
         <v>205</v>
       </c>
-      <c r="O7" s="63">
+      <c r="O7" s="16">
         <v>251</v>
       </c>
     </row>
@@ -3886,13 +3886,13 @@
       <c r="G8" s="1">
         <v>77</v>
       </c>
-      <c r="I8" s="62">
+      <c r="I8" s="15">
         <v>6</v>
       </c>
-      <c r="J8" s="63">
+      <c r="J8" s="16">
         <v>15</v>
       </c>
-      <c r="L8" s="62">
+      <c r="L8" s="15">
         <v>624</v>
       </c>
       <c r="M8" s="2">
@@ -3901,7 +3901,7 @@
       <c r="N8" s="2">
         <v>338</v>
       </c>
-      <c r="O8" s="63">
+      <c r="O8" s="16">
         <v>440</v>
       </c>
     </row>
@@ -3926,13 +3926,13 @@
       <c r="G9" s="1">
         <v>60</v>
       </c>
-      <c r="I9" s="62">
+      <c r="I9" s="15">
         <v>7</v>
       </c>
-      <c r="J9" s="63">
+      <c r="J9" s="16">
         <v>18</v>
       </c>
-      <c r="L9" s="62">
+      <c r="L9" s="15">
         <v>7200</v>
       </c>
       <c r="M9" s="2">
@@ -3941,7 +3941,7 @@
       <c r="N9" s="2">
         <v>797</v>
       </c>
-      <c r="O9" s="63">
+      <c r="O9" s="16">
         <v>1003</v>
       </c>
     </row>
@@ -3966,13 +3966,13 @@
       <c r="G10" s="1">
         <v>132</v>
       </c>
-      <c r="I10" s="62">
+      <c r="I10" s="15">
         <v>8</v>
       </c>
-      <c r="J10" s="63">
+      <c r="J10" s="16">
         <v>21</v>
       </c>
-      <c r="L10" s="62">
+      <c r="L10" s="15">
         <v>1472</v>
       </c>
       <c r="M10" s="2">
@@ -3981,7 +3981,7 @@
       <c r="N10" s="2">
         <v>1340</v>
       </c>
-      <c r="O10" s="63">
+      <c r="O10" s="16">
         <v>1272</v>
       </c>
     </row>
@@ -4006,13 +4006,13 @@
       <c r="G11" s="1">
         <v>99</v>
       </c>
-      <c r="I11" s="62">
+      <c r="I11" s="15">
         <v>9</v>
       </c>
-      <c r="J11" s="63">
+      <c r="J11" s="16">
         <v>24</v>
       </c>
-      <c r="L11" s="62">
+      <c r="L11" s="15">
         <v>7200</v>
       </c>
       <c r="M11" s="2">
@@ -4021,7 +4021,7 @@
       <c r="N11" s="2">
         <v>1700</v>
       </c>
-      <c r="O11" s="63">
+      <c r="O11" s="16">
         <v>2556</v>
       </c>
     </row>
@@ -4046,13 +4046,13 @@
       <c r="G12" s="1">
         <v>205</v>
       </c>
-      <c r="I12" s="62">
+      <c r="I12" s="15">
         <v>10</v>
       </c>
-      <c r="J12" s="63">
+      <c r="J12" s="16">
         <v>27</v>
       </c>
-      <c r="L12" s="62">
+      <c r="L12" s="15">
         <v>7200</v>
       </c>
       <c r="M12" s="2">
@@ -4061,7 +4061,7 @@
       <c r="N12" s="2">
         <v>3241</v>
       </c>
-      <c r="O12" s="63">
+      <c r="O12" s="16">
         <v>3494</v>
       </c>
     </row>
@@ -4086,13 +4086,13 @@
       <c r="G13" s="1">
         <v>251</v>
       </c>
-      <c r="I13" s="62">
+      <c r="I13" s="15">
         <v>11</v>
       </c>
-      <c r="J13" s="63">
+      <c r="J13" s="16">
         <v>30</v>
       </c>
-      <c r="L13" s="62">
+      <c r="L13" s="15">
         <v>7200</v>
       </c>
       <c r="M13" s="2">
@@ -4101,7 +4101,7 @@
       <c r="N13" s="2">
         <v>7200</v>
       </c>
-      <c r="O13" s="63">
+      <c r="O13" s="16">
         <v>4905</v>
       </c>
     </row>
@@ -4126,13 +4126,13 @@
       <c r="G14" s="1">
         <v>624</v>
       </c>
-      <c r="I14" s="62">
+      <c r="I14" s="15">
         <v>12</v>
       </c>
-      <c r="J14" s="63">
+      <c r="J14" s="16">
         <v>33</v>
       </c>
-      <c r="L14" s="62">
+      <c r="L14" s="15">
         <v>7200</v>
       </c>
       <c r="M14" s="2">
@@ -4141,7 +4141,7 @@
       <c r="N14" s="5">
         <v>6908</v>
       </c>
-      <c r="O14" s="63">
+      <c r="O14" s="16">
         <v>7200</v>
       </c>
     </row>
@@ -4166,22 +4166,22 @@
       <c r="G15" s="1">
         <v>239</v>
       </c>
-      <c r="I15" s="64">
+      <c r="I15" s="17">
         <v>13</v>
       </c>
-      <c r="J15" s="65">
+      <c r="J15" s="18">
         <v>36</v>
       </c>
-      <c r="L15" s="64">
+      <c r="L15" s="17">
         <v>7200</v>
       </c>
-      <c r="M15" s="70">
+      <c r="M15" s="23">
         <v>7200</v>
       </c>
-      <c r="N15" s="70">
+      <c r="N15" s="23">
         <v>7200</v>
       </c>
-      <c r="O15" s="65">
+      <c r="O15" s="18">
         <v>7200</v>
       </c>
     </row>
@@ -5222,708 +5222,791 @@
       </c>
     </row>
     <row r="3" spans="2:20" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="44" t="s">
+      <c r="B3" s="72" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="16"/>
-      <c r="D3" s="45" t="s">
+      <c r="C3" s="29"/>
+      <c r="D3" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="E3" s="46" t="s">
+      <c r="E3" s="73" t="s">
         <v>48</v>
       </c>
-      <c r="F3" s="33" t="s">
+      <c r="F3" s="37" t="s">
         <v>51</v>
       </c>
-      <c r="G3" s="40" t="s">
+      <c r="G3" s="50" t="s">
         <v>76</v>
       </c>
-      <c r="H3" s="19" t="s">
+      <c r="H3" s="45" t="s">
         <v>77</v>
       </c>
-      <c r="I3" s="19"/>
-      <c r="J3" s="19"/>
-      <c r="K3" s="33" t="s">
+      <c r="I3" s="45"/>
+      <c r="J3" s="45"/>
+      <c r="K3" s="37" t="s">
         <v>78</v>
       </c>
-      <c r="L3" s="40" t="s">
+      <c r="L3" s="50" t="s">
         <v>79</v>
       </c>
-      <c r="M3" s="42" t="s">
+      <c r="M3" s="62" t="s">
         <v>53</v>
       </c>
-      <c r="N3" s="33" t="s">
+      <c r="N3" s="37" t="s">
         <v>80</v>
       </c>
       <c r="O3" s="13"/>
     </row>
     <row r="4" spans="2:20" ht="10.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="35"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="46"/>
-      <c r="F4" s="33"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="20"/>
-      <c r="I4" s="20"/>
-      <c r="J4" s="20"/>
-      <c r="K4" s="34"/>
-      <c r="L4" s="41"/>
-      <c r="M4" s="43"/>
-      <c r="N4" s="34"/>
+      <c r="B4" s="33"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="73"/>
+      <c r="F4" s="37"/>
+      <c r="G4" s="35"/>
+      <c r="H4" s="74"/>
+      <c r="I4" s="74"/>
+      <c r="J4" s="74"/>
+      <c r="K4" s="47"/>
+      <c r="L4" s="35"/>
+      <c r="M4" s="60"/>
+      <c r="N4" s="47"/>
       <c r="O4" s="13"/>
     </row>
     <row r="5" spans="2:20" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="35" t="s">
+      <c r="B5" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="36" t="s">
+      <c r="C5" s="38" t="s">
         <v>81</v>
       </c>
-      <c r="D5" s="38" t="s">
+      <c r="D5" s="63" t="s">
         <v>82</v>
       </c>
-      <c r="E5" s="36" t="s">
+      <c r="E5" s="38" t="s">
         <v>83</v>
       </c>
-      <c r="F5" s="47"/>
-      <c r="G5" s="45" t="s">
+      <c r="F5" s="36"/>
+      <c r="G5" s="34" t="s">
         <v>47</v>
       </c>
-      <c r="H5" s="36"/>
-      <c r="I5" s="21" t="s">
+      <c r="H5" s="38"/>
+      <c r="I5" s="66" t="s">
         <v>48</v>
       </c>
-      <c r="J5" s="21"/>
-      <c r="K5" s="21"/>
-      <c r="L5" s="47" t="s">
+      <c r="J5" s="66"/>
+      <c r="K5" s="66"/>
+      <c r="L5" s="36" t="s">
         <v>49</v>
       </c>
       <c r="N5" s="14"/>
       <c r="O5" s="13"/>
     </row>
     <row r="6" spans="2:20" ht="10.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="35"/>
-      <c r="C6" s="37"/>
-      <c r="D6" s="39"/>
-      <c r="E6" s="37"/>
-      <c r="F6" s="34"/>
-      <c r="G6" s="41"/>
-      <c r="H6" s="37"/>
-      <c r="I6" s="22"/>
-      <c r="J6" s="22"/>
-      <c r="K6" s="22"/>
-      <c r="L6" s="34"/>
+      <c r="B6" s="33"/>
+      <c r="C6" s="39"/>
+      <c r="D6" s="64"/>
+      <c r="E6" s="39"/>
+      <c r="F6" s="47"/>
+      <c r="G6" s="35"/>
+      <c r="H6" s="39"/>
+      <c r="I6" s="75"/>
+      <c r="J6" s="75"/>
+      <c r="K6" s="75"/>
+      <c r="L6" s="47"/>
       <c r="N6" s="14"/>
       <c r="O6" s="13"/>
     </row>
     <row r="7" spans="2:20" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="35" t="s">
+      <c r="B7" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="D7" s="45" t="s">
+      <c r="D7" s="34" t="s">
         <v>84</v>
       </c>
-      <c r="E7" s="36"/>
-      <c r="F7" s="38" t="s">
+      <c r="E7" s="38"/>
+      <c r="F7" s="63" t="s">
         <v>82</v>
       </c>
-      <c r="G7" s="36" t="s">
+      <c r="G7" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="H7" s="47"/>
-      <c r="I7" s="45" t="s">
+      <c r="H7" s="36"/>
+      <c r="I7" s="34" t="s">
         <v>86</v>
       </c>
-      <c r="J7" s="23" t="s">
+      <c r="J7" s="40" t="s">
         <v>87</v>
       </c>
-      <c r="K7" s="23"/>
-      <c r="L7" s="47" t="s">
+      <c r="K7" s="40"/>
+      <c r="L7" s="36" t="s">
         <v>88</v>
       </c>
       <c r="N7" s="14"/>
       <c r="O7" s="13"/>
     </row>
     <row r="8" spans="2:20" ht="10.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="35"/>
-      <c r="D8" s="41"/>
-      <c r="E8" s="37"/>
-      <c r="F8" s="48"/>
-      <c r="G8" s="37"/>
-      <c r="H8" s="34"/>
-      <c r="I8" s="41"/>
-      <c r="J8" s="24"/>
-      <c r="K8" s="24"/>
-      <c r="L8" s="33"/>
+      <c r="B8" s="33"/>
+      <c r="D8" s="35"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="71"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="47"/>
+      <c r="I8" s="35"/>
+      <c r="J8" s="41"/>
+      <c r="K8" s="41"/>
+      <c r="L8" s="37"/>
       <c r="N8" s="14"/>
       <c r="O8" s="13"/>
     </row>
     <row r="9" spans="2:20" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="35" t="s">
+      <c r="B9" s="33" t="s">
         <v>43</v>
       </c>
-      <c r="C9" s="36" t="s">
+      <c r="C9" s="38" t="s">
         <v>89</v>
       </c>
-      <c r="D9" s="27" t="s">
+      <c r="D9" s="48" t="s">
         <v>90</v>
       </c>
-      <c r="E9" s="27"/>
-      <c r="F9" s="47" t="s">
+      <c r="E9" s="48"/>
+      <c r="F9" s="36" t="s">
         <v>91</v>
       </c>
-      <c r="G9" s="45" t="s">
+      <c r="G9" s="34" t="s">
         <v>92</v>
       </c>
-      <c r="H9" s="25" t="s">
+      <c r="H9" s="57" t="s">
         <v>59</v>
       </c>
-      <c r="I9" s="25"/>
-      <c r="J9" s="25"/>
-      <c r="K9" s="47" t="s">
+      <c r="I9" s="57"/>
+      <c r="J9" s="57"/>
+      <c r="K9" s="36" t="s">
         <v>93</v>
       </c>
-      <c r="L9" s="45" t="s">
+      <c r="L9" s="34" t="s">
         <v>94</v>
       </c>
-      <c r="M9" s="49" t="s">
+      <c r="M9" s="55" t="s">
         <v>95</v>
       </c>
-      <c r="N9" s="47" t="s">
+      <c r="N9" s="36" t="s">
         <v>96</v>
       </c>
       <c r="O9" s="13"/>
     </row>
     <row r="10" spans="2:20" ht="10.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="35"/>
-      <c r="C10" s="37"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="28"/>
-      <c r="F10" s="34"/>
-      <c r="G10" s="41"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="26"/>
-      <c r="J10" s="26"/>
-      <c r="K10" s="34"/>
-      <c r="L10" s="41"/>
-      <c r="M10" s="50"/>
-      <c r="N10" s="34"/>
+      <c r="B10" s="33"/>
+      <c r="C10" s="39"/>
+      <c r="D10" s="49"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="47"/>
+      <c r="G10" s="35"/>
+      <c r="H10" s="58"/>
+      <c r="I10" s="58"/>
+      <c r="J10" s="58"/>
+      <c r="K10" s="47"/>
+      <c r="L10" s="35"/>
+      <c r="M10" s="56"/>
+      <c r="N10" s="47"/>
       <c r="O10" s="13"/>
     </row>
     <row r="11" spans="2:20" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="35" t="s">
+      <c r="B11" s="33" t="s">
         <v>97</v>
       </c>
-      <c r="D11" s="45" t="s">
+      <c r="D11" s="34" t="s">
         <v>54</v>
       </c>
-      <c r="E11" s="29" t="s">
+      <c r="E11" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="F11" s="29"/>
-      <c r="G11" s="29"/>
-      <c r="H11" s="47" t="s">
+      <c r="F11" s="68"/>
+      <c r="G11" s="68"/>
+      <c r="H11" s="36" t="s">
         <v>55</v>
       </c>
-      <c r="I11" s="45" t="s">
+      <c r="I11" s="34" t="s">
         <v>98</v>
       </c>
-      <c r="J11" s="52" t="s">
+      <c r="J11" s="42" t="s">
         <v>99</v>
       </c>
-      <c r="K11" s="36" t="s">
+      <c r="K11" s="38" t="s">
         <v>100</v>
       </c>
-      <c r="L11" s="47"/>
-      <c r="M11" s="16"/>
-      <c r="N11" s="51"/>
+      <c r="L11" s="36"/>
+      <c r="M11" s="29"/>
+      <c r="N11" s="61"/>
       <c r="O11" s="13"/>
     </row>
     <row r="12" spans="2:20" ht="10.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="35"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="30"/>
-      <c r="F12" s="30"/>
-      <c r="G12" s="30"/>
-      <c r="H12" s="34"/>
-      <c r="I12" s="41"/>
-      <c r="J12" s="53"/>
-      <c r="K12" s="37"/>
-      <c r="L12" s="34"/>
-      <c r="M12" s="16"/>
-      <c r="N12" s="51"/>
+      <c r="B12" s="33"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="69"/>
+      <c r="F12" s="69"/>
+      <c r="G12" s="69"/>
+      <c r="H12" s="47"/>
+      <c r="I12" s="35"/>
+      <c r="J12" s="43"/>
+      <c r="K12" s="39"/>
+      <c r="L12" s="47"/>
+      <c r="M12" s="29"/>
+      <c r="N12" s="61"/>
       <c r="O12" s="13"/>
     </row>
     <row r="13" spans="2:20" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="35" t="s">
+      <c r="B13" s="33" t="s">
         <v>101</v>
       </c>
-      <c r="E13" s="45" t="s">
+      <c r="E13" s="34" t="s">
         <v>102</v>
       </c>
-      <c r="F13" s="36"/>
-      <c r="G13" s="31" t="s">
+      <c r="F13" s="38"/>
+      <c r="G13" s="53" t="s">
         <v>103</v>
       </c>
-      <c r="H13" s="31"/>
-      <c r="I13" s="31"/>
-      <c r="J13" s="47" t="s">
+      <c r="H13" s="53"/>
+      <c r="I13" s="53"/>
+      <c r="J13" s="36" t="s">
         <v>104</v>
       </c>
-      <c r="K13" s="45" t="s">
+      <c r="K13" s="34" t="s">
         <v>105</v>
       </c>
-      <c r="L13" s="25" t="s">
+      <c r="L13" s="57" t="s">
         <v>59</v>
       </c>
-      <c r="M13" s="25"/>
-      <c r="N13" s="25"/>
-      <c r="O13" s="47" t="s">
+      <c r="M13" s="57"/>
+      <c r="N13" s="57"/>
+      <c r="O13" s="36" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="14" spans="2:20" ht="10.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="35"/>
-      <c r="E14" s="41"/>
-      <c r="F14" s="37"/>
-      <c r="G14" s="32"/>
-      <c r="H14" s="32"/>
-      <c r="I14" s="32"/>
-      <c r="J14" s="34"/>
-      <c r="K14" s="41"/>
-      <c r="L14" s="26"/>
-      <c r="M14" s="26"/>
-      <c r="N14" s="26"/>
-      <c r="O14" s="34"/>
+      <c r="B14" s="33"/>
+      <c r="E14" s="35"/>
+      <c r="F14" s="39"/>
+      <c r="G14" s="54"/>
+      <c r="H14" s="54"/>
+      <c r="I14" s="54"/>
+      <c r="J14" s="47"/>
+      <c r="K14" s="35"/>
+      <c r="L14" s="58"/>
+      <c r="M14" s="58"/>
+      <c r="N14" s="58"/>
+      <c r="O14" s="47"/>
     </row>
     <row r="15" spans="2:20" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="35" t="s">
+      <c r="B15" s="33" t="s">
         <v>107</v>
       </c>
-      <c r="E15" s="45" t="s">
+      <c r="E15" s="34" t="s">
         <v>108</v>
       </c>
-      <c r="F15" s="21" t="s">
+      <c r="F15" s="66" t="s">
         <v>48</v>
       </c>
-      <c r="G15" s="47" t="s">
+      <c r="G15" s="36" t="s">
         <v>109</v>
       </c>
-      <c r="H15" s="45" t="s">
+      <c r="H15" s="34" t="s">
         <v>110</v>
       </c>
-      <c r="I15" s="29" t="s">
+      <c r="I15" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="J15" s="29" t="s">
+      <c r="J15" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="K15" s="29"/>
-      <c r="L15" s="55" t="s">
+      <c r="K15" s="68"/>
+      <c r="L15" s="70" t="s">
         <v>46</v>
       </c>
-      <c r="M15" s="36" t="s">
+      <c r="M15" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="N15" s="47"/>
+      <c r="N15" s="36"/>
       <c r="O15" s="13"/>
     </row>
     <row r="16" spans="2:20" ht="10.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="35"/>
-      <c r="E16" s="40"/>
-      <c r="F16" s="54"/>
-      <c r="G16" s="34"/>
-      <c r="H16" s="41"/>
-      <c r="I16" s="30"/>
-      <c r="J16" s="56" t="s">
+      <c r="B16" s="33"/>
+      <c r="E16" s="50"/>
+      <c r="F16" s="67"/>
+      <c r="G16" s="47"/>
+      <c r="H16" s="35"/>
+      <c r="I16" s="69"/>
+      <c r="J16" s="52" t="s">
         <v>112</v>
       </c>
-      <c r="K16" s="56"/>
-      <c r="L16" s="30"/>
-      <c r="M16" s="37"/>
-      <c r="N16" s="34"/>
+      <c r="K16" s="52"/>
+      <c r="L16" s="69"/>
+      <c r="M16" s="39"/>
+      <c r="N16" s="47"/>
       <c r="O16" s="13"/>
     </row>
     <row r="17" spans="2:15" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="35" t="s">
+      <c r="B17" s="33" t="s">
         <v>113</v>
       </c>
-      <c r="D17" s="45" t="s">
+      <c r="D17" s="34" t="s">
         <v>114</v>
       </c>
-      <c r="E17" s="38" t="s">
+      <c r="E17" s="63" t="s">
         <v>82</v>
       </c>
-      <c r="F17" s="47" t="s">
+      <c r="F17" s="36" t="s">
         <v>115</v>
       </c>
-      <c r="G17" s="45" t="s">
+      <c r="G17" s="34" t="s">
         <v>116</v>
       </c>
-      <c r="H17" s="52" t="s">
+      <c r="H17" s="42" t="s">
         <v>99</v>
       </c>
-      <c r="I17" s="52"/>
-      <c r="J17" s="47" t="s">
+      <c r="I17" s="42"/>
+      <c r="J17" s="36" t="s">
         <v>117</v>
       </c>
-      <c r="K17" s="45" t="s">
+      <c r="K17" s="34" t="s">
         <v>118</v>
       </c>
-      <c r="L17" s="49" t="s">
+      <c r="L17" s="55" t="s">
         <v>95</v>
       </c>
-      <c r="M17" s="36" t="s">
+      <c r="M17" s="38" t="s">
         <v>119</v>
       </c>
-      <c r="N17" s="47"/>
+      <c r="N17" s="36"/>
       <c r="O17" s="13"/>
     </row>
     <row r="18" spans="2:15" ht="10.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="35"/>
-      <c r="D18" s="41"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="34"/>
-      <c r="G18" s="41"/>
-      <c r="H18" s="53"/>
-      <c r="I18" s="53"/>
-      <c r="J18" s="34"/>
-      <c r="K18" s="41"/>
-      <c r="L18" s="57"/>
-      <c r="M18" s="37"/>
-      <c r="N18" s="34"/>
+      <c r="B18" s="33"/>
+      <c r="D18" s="35"/>
+      <c r="E18" s="64"/>
+      <c r="F18" s="47"/>
+      <c r="G18" s="35"/>
+      <c r="H18" s="43"/>
+      <c r="I18" s="43"/>
+      <c r="J18" s="47"/>
+      <c r="K18" s="35"/>
+      <c r="L18" s="65"/>
+      <c r="M18" s="39"/>
+      <c r="N18" s="47"/>
       <c r="O18" s="13"/>
     </row>
     <row r="19" spans="2:15" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="35" t="s">
+      <c r="B19" s="33" t="s">
         <v>120</v>
       </c>
-      <c r="D19" s="45" t="s">
+      <c r="D19" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="E19" s="36"/>
-      <c r="F19" s="58" t="s">
+      <c r="E19" s="38"/>
+      <c r="F19" s="59" t="s">
         <v>53</v>
       </c>
       <c r="G19" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="H19" s="58" t="s">
+      <c r="H19" s="59" t="s">
         <v>53</v>
       </c>
-      <c r="I19" s="47" t="s">
+      <c r="I19" s="36" t="s">
         <v>57</v>
       </c>
-      <c r="J19" s="45" t="s">
+      <c r="J19" s="34" t="s">
         <v>121</v>
       </c>
-      <c r="K19" s="31" t="s">
+      <c r="K19" s="53" t="s">
         <v>103</v>
       </c>
-      <c r="L19" s="31"/>
-      <c r="M19" s="47" t="s">
+      <c r="L19" s="53"/>
+      <c r="M19" s="36" t="s">
         <v>122</v>
       </c>
-      <c r="N19" s="51"/>
+      <c r="N19" s="61"/>
       <c r="O19" s="13"/>
     </row>
     <row r="20" spans="2:15" ht="10.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="35"/>
-      <c r="D20" s="41"/>
-      <c r="E20" s="37"/>
-      <c r="F20" s="42"/>
+      <c r="B20" s="33"/>
+      <c r="D20" s="35"/>
+      <c r="E20" s="39"/>
+      <c r="F20" s="62"/>
       <c r="G20" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="H20" s="43"/>
-      <c r="I20" s="34"/>
-      <c r="J20" s="41"/>
-      <c r="K20" s="32"/>
-      <c r="L20" s="32"/>
-      <c r="M20" s="34"/>
-      <c r="N20" s="51"/>
+      <c r="H20" s="60"/>
+      <c r="I20" s="47"/>
+      <c r="J20" s="35"/>
+      <c r="K20" s="54"/>
+      <c r="L20" s="54"/>
+      <c r="M20" s="47"/>
+      <c r="N20" s="61"/>
       <c r="O20" s="13"/>
     </row>
     <row r="21" spans="2:15" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="35" t="s">
+      <c r="B21" s="33" t="s">
         <v>123</v>
       </c>
-      <c r="C21" s="36" t="s">
+      <c r="C21" s="38" t="s">
         <v>61</v>
       </c>
-      <c r="D21" s="25" t="s">
+      <c r="D21" s="57" t="s">
         <v>59</v>
       </c>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="47" t="s">
+      <c r="E21" s="57"/>
+      <c r="F21" s="57"/>
+      <c r="G21" s="36" t="s">
         <v>62</v>
       </c>
-      <c r="H21" s="16"/>
-      <c r="I21" s="45" t="s">
+      <c r="H21" s="29"/>
+      <c r="I21" s="34" t="s">
         <v>52</v>
       </c>
-      <c r="J21" s="58" t="s">
+      <c r="J21" s="59" t="s">
         <v>53</v>
       </c>
-      <c r="K21" s="58"/>
-      <c r="L21" s="58"/>
-      <c r="M21" s="47" t="s">
+      <c r="K21" s="59"/>
+      <c r="L21" s="59"/>
+      <c r="M21" s="36" t="s">
         <v>124</v>
       </c>
-      <c r="N21" s="51"/>
+      <c r="N21" s="61"/>
       <c r="O21" s="13"/>
     </row>
     <row r="22" spans="2:15" ht="10.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="35"/>
-      <c r="C22" s="37"/>
-      <c r="D22" s="26"/>
-      <c r="E22" s="26"/>
-      <c r="F22" s="26"/>
-      <c r="G22" s="33"/>
-      <c r="H22" s="16"/>
-      <c r="I22" s="40"/>
-      <c r="J22" s="43"/>
-      <c r="K22" s="43"/>
-      <c r="L22" s="43"/>
-      <c r="M22" s="33"/>
-      <c r="N22" s="51"/>
+      <c r="B22" s="33"/>
+      <c r="C22" s="39"/>
+      <c r="D22" s="58"/>
+      <c r="E22" s="58"/>
+      <c r="F22" s="58"/>
+      <c r="G22" s="37"/>
+      <c r="H22" s="29"/>
+      <c r="I22" s="50"/>
+      <c r="J22" s="60"/>
+      <c r="K22" s="60"/>
+      <c r="L22" s="60"/>
+      <c r="M22" s="37"/>
+      <c r="N22" s="61"/>
       <c r="O22" s="13"/>
     </row>
     <row r="23" spans="2:15" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="35" t="s">
+      <c r="B23" s="33" t="s">
         <v>125</v>
       </c>
-      <c r="D23" s="16"/>
-      <c r="E23" s="45" t="s">
+      <c r="D23" s="29"/>
+      <c r="E23" s="34" t="s">
         <v>126</v>
       </c>
-      <c r="F23" s="36"/>
-      <c r="G23" s="27" t="s">
+      <c r="F23" s="38"/>
+      <c r="G23" s="48" t="s">
         <v>90</v>
       </c>
-      <c r="H23" s="27"/>
-      <c r="I23" s="27"/>
-      <c r="J23" s="47" t="s">
+      <c r="H23" s="48"/>
+      <c r="I23" s="48"/>
+      <c r="J23" s="36" t="s">
         <v>127</v>
       </c>
-      <c r="K23" s="45" t="s">
+      <c r="K23" s="34" t="s">
         <v>128</v>
       </c>
-      <c r="L23" s="23" t="s">
+      <c r="L23" s="40" t="s">
         <v>87</v>
       </c>
-      <c r="M23" s="23"/>
-      <c r="N23" s="36" t="s">
+      <c r="M23" s="40"/>
+      <c r="N23" s="38" t="s">
         <v>129</v>
       </c>
-      <c r="O23" s="47"/>
+      <c r="O23" s="36"/>
     </row>
     <row r="24" spans="2:15" ht="10.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="35"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="41"/>
-      <c r="F24" s="37"/>
-      <c r="G24" s="28"/>
-      <c r="H24" s="28"/>
-      <c r="I24" s="28"/>
-      <c r="J24" s="34"/>
-      <c r="K24" s="41"/>
-      <c r="L24" s="24"/>
-      <c r="M24" s="24"/>
-      <c r="N24" s="37"/>
-      <c r="O24" s="34"/>
+      <c r="B24" s="33"/>
+      <c r="D24" s="29"/>
+      <c r="E24" s="35"/>
+      <c r="F24" s="39"/>
+      <c r="G24" s="49"/>
+      <c r="H24" s="49"/>
+      <c r="I24" s="49"/>
+      <c r="J24" s="47"/>
+      <c r="K24" s="35"/>
+      <c r="L24" s="41"/>
+      <c r="M24" s="41"/>
+      <c r="N24" s="39"/>
+      <c r="O24" s="47"/>
     </row>
     <row r="25" spans="2:15" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="35" t="s">
+      <c r="B25" s="33" t="s">
         <v>130</v>
       </c>
-      <c r="D25" s="16"/>
-      <c r="E25" s="45" t="s">
+      <c r="D25" s="29"/>
+      <c r="E25" s="34" t="s">
         <v>131</v>
       </c>
-      <c r="F25" s="59" t="s">
+      <c r="F25" s="51" t="s">
         <v>112</v>
       </c>
-      <c r="G25" s="59"/>
-      <c r="H25" s="59"/>
-      <c r="I25" s="36" t="s">
+      <c r="G25" s="51"/>
+      <c r="H25" s="51"/>
+      <c r="I25" s="38" t="s">
         <v>132</v>
       </c>
-      <c r="J25" s="47"/>
-      <c r="K25" s="45" t="s">
+      <c r="J25" s="36"/>
+      <c r="K25" s="34" t="s">
         <v>133</v>
       </c>
-      <c r="L25" s="36"/>
-      <c r="M25" s="31" t="s">
+      <c r="L25" s="38"/>
+      <c r="M25" s="53" t="s">
         <v>103</v>
       </c>
-      <c r="N25" s="47" t="s">
+      <c r="N25" s="36" t="s">
         <v>134</v>
       </c>
       <c r="O25" s="13"/>
     </row>
     <row r="26" spans="2:15" ht="10.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="35"/>
-      <c r="D26" s="16"/>
-      <c r="E26" s="40"/>
-      <c r="F26" s="56"/>
-      <c r="G26" s="56"/>
-      <c r="H26" s="56"/>
-      <c r="I26" s="37"/>
-      <c r="J26" s="34"/>
-      <c r="K26" s="41"/>
-      <c r="L26" s="37"/>
-      <c r="M26" s="32"/>
-      <c r="N26" s="34"/>
+      <c r="B26" s="33"/>
+      <c r="D26" s="29"/>
+      <c r="E26" s="50"/>
+      <c r="F26" s="52"/>
+      <c r="G26" s="52"/>
+      <c r="H26" s="52"/>
+      <c r="I26" s="39"/>
+      <c r="J26" s="47"/>
+      <c r="K26" s="35"/>
+      <c r="L26" s="39"/>
+      <c r="M26" s="54"/>
+      <c r="N26" s="47"/>
       <c r="O26" s="13"/>
     </row>
     <row r="27" spans="2:15" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="35" t="s">
+      <c r="B27" s="33" t="s">
         <v>135</v>
       </c>
-      <c r="D27" s="45" t="s">
+      <c r="D27" s="34" t="s">
         <v>136</v>
       </c>
-      <c r="E27" s="19" t="s">
+      <c r="E27" s="45" t="s">
         <v>77</v>
       </c>
-      <c r="F27" s="47" t="s">
+      <c r="F27" s="36" t="s">
         <v>137</v>
       </c>
-      <c r="G27" s="45" t="s">
+      <c r="G27" s="34" t="s">
         <v>138</v>
       </c>
-      <c r="H27" s="49" t="s">
+      <c r="H27" s="55" t="s">
         <v>95</v>
       </c>
-      <c r="I27" s="49"/>
-      <c r="J27" s="49"/>
-      <c r="K27" s="47" t="s">
+      <c r="I27" s="55"/>
+      <c r="J27" s="55"/>
+      <c r="K27" s="36" t="s">
         <v>139</v>
       </c>
-      <c r="L27" s="16"/>
-      <c r="M27" s="16"/>
+      <c r="L27" s="29"/>
+      <c r="M27" s="29"/>
       <c r="N27" s="14"/>
       <c r="O27" s="13"/>
     </row>
     <row r="28" spans="2:15" ht="10.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="35"/>
-      <c r="D28" s="41"/>
-      <c r="E28" s="60"/>
-      <c r="F28" s="34"/>
-      <c r="G28" s="41"/>
-      <c r="H28" s="50"/>
-      <c r="I28" s="50"/>
-      <c r="J28" s="50"/>
-      <c r="K28" s="33"/>
-      <c r="L28" s="16"/>
-      <c r="M28" s="16"/>
+      <c r="B28" s="33"/>
+      <c r="D28" s="35"/>
+      <c r="E28" s="46"/>
+      <c r="F28" s="47"/>
+      <c r="G28" s="35"/>
+      <c r="H28" s="56"/>
+      <c r="I28" s="56"/>
+      <c r="J28" s="56"/>
+      <c r="K28" s="37"/>
+      <c r="L28" s="29"/>
+      <c r="M28" s="29"/>
       <c r="N28" s="14"/>
       <c r="O28" s="13"/>
     </row>
     <row r="29" spans="2:15" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="35" t="s">
+      <c r="B29" s="33" t="s">
         <v>140</v>
       </c>
-      <c r="E29" s="45" t="s">
+      <c r="E29" s="34" t="s">
         <v>141</v>
       </c>
-      <c r="F29" s="23" t="s">
+      <c r="F29" s="40" t="s">
         <v>87</v>
       </c>
-      <c r="G29" s="23"/>
-      <c r="H29" s="23"/>
-      <c r="I29" s="47" t="s">
+      <c r="G29" s="40"/>
+      <c r="H29" s="40"/>
+      <c r="I29" s="36" t="s">
         <v>142</v>
       </c>
-      <c r="J29" s="45" t="s">
+      <c r="J29" s="34" t="s">
         <v>143</v>
       </c>
-      <c r="K29" s="36"/>
-      <c r="L29" s="52" t="s">
+      <c r="K29" s="38"/>
+      <c r="L29" s="42" t="s">
         <v>99</v>
       </c>
-      <c r="M29" s="52"/>
-      <c r="N29" s="47" t="s">
+      <c r="M29" s="42"/>
+      <c r="N29" s="36" t="s">
         <v>144</v>
       </c>
       <c r="O29" s="13"/>
     </row>
     <row r="30" spans="2:15" ht="10.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="35"/>
-      <c r="E30" s="41"/>
-      <c r="F30" s="24"/>
-      <c r="G30" s="24"/>
-      <c r="H30" s="24"/>
-      <c r="I30" s="33"/>
-      <c r="J30" s="41"/>
-      <c r="K30" s="37"/>
-      <c r="L30" s="53"/>
-      <c r="M30" s="53"/>
-      <c r="N30" s="33"/>
+      <c r="B30" s="33"/>
+      <c r="E30" s="35"/>
+      <c r="F30" s="41"/>
+      <c r="G30" s="41"/>
+      <c r="H30" s="41"/>
+      <c r="I30" s="37"/>
+      <c r="J30" s="35"/>
+      <c r="K30" s="39"/>
+      <c r="L30" s="43"/>
+      <c r="M30" s="43"/>
+      <c r="N30" s="37"/>
       <c r="O30" s="13"/>
     </row>
     <row r="31" spans="2:15" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="35" t="s">
+      <c r="B31" s="33" t="s">
         <v>145</v>
       </c>
-      <c r="F31" s="45" t="s">
+      <c r="F31" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="G31" s="19" t="s">
+      <c r="G31" s="45" t="s">
         <v>77</v>
       </c>
-      <c r="H31" s="47" t="s">
+      <c r="H31" s="36" t="s">
         <v>60</v>
       </c>
-      <c r="I31" s="45" t="s">
+      <c r="I31" s="34" t="s">
         <v>146</v>
       </c>
-      <c r="J31" s="36"/>
-      <c r="K31" s="27" t="s">
+      <c r="J31" s="38"/>
+      <c r="K31" s="48" t="s">
         <v>90</v>
       </c>
-      <c r="L31" s="27"/>
-      <c r="M31" s="27"/>
-      <c r="N31" s="36" t="s">
+      <c r="L31" s="48"/>
+      <c r="M31" s="48"/>
+      <c r="N31" s="38" t="s">
         <v>147</v>
       </c>
-      <c r="O31" s="47"/>
+      <c r="O31" s="36"/>
     </row>
     <row r="32" spans="2:15" ht="10.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="61"/>
+      <c r="B32" s="44"/>
       <c r="C32" s="7"/>
       <c r="D32" s="7"/>
       <c r="E32" s="7"/>
-      <c r="F32" s="41"/>
-      <c r="G32" s="60"/>
-      <c r="H32" s="34"/>
-      <c r="I32" s="41"/>
-      <c r="J32" s="37"/>
-      <c r="K32" s="28"/>
-      <c r="L32" s="28"/>
-      <c r="M32" s="28"/>
-      <c r="N32" s="37"/>
-      <c r="O32" s="34"/>
+      <c r="F32" s="35"/>
+      <c r="G32" s="46"/>
+      <c r="H32" s="47"/>
+      <c r="I32" s="35"/>
+      <c r="J32" s="39"/>
+      <c r="K32" s="49"/>
+      <c r="L32" s="49"/>
+      <c r="M32" s="49"/>
+      <c r="N32" s="39"/>
+      <c r="O32" s="47"/>
     </row>
   </sheetData>
   <mergeCells count="128">
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="I29:I30"/>
-    <mergeCell ref="J29:K30"/>
-    <mergeCell ref="F29:H30"/>
-    <mergeCell ref="L29:M30"/>
-    <mergeCell ref="N29:N30"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="G31:G32"/>
-    <mergeCell ref="H31:H32"/>
-    <mergeCell ref="I31:J32"/>
-    <mergeCell ref="N31:O32"/>
-    <mergeCell ref="K31:M32"/>
+    <mergeCell ref="N3:N4"/>
+    <mergeCell ref="M9:M10"/>
+    <mergeCell ref="N9:N10"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="L3:L4"/>
+    <mergeCell ref="M3:M4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="G5:H6"/>
+    <mergeCell ref="E5:F6"/>
+    <mergeCell ref="L5:L6"/>
+    <mergeCell ref="H3:J4"/>
+    <mergeCell ref="I5:K6"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="D7:E8"/>
+    <mergeCell ref="G7:H8"/>
+    <mergeCell ref="L7:L8"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="J7:K8"/>
+    <mergeCell ref="H9:J10"/>
+    <mergeCell ref="D9:E10"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="K11:L12"/>
+    <mergeCell ref="N11:N12"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="K13:K14"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="M11:M12"/>
+    <mergeCell ref="E13:F14"/>
+    <mergeCell ref="E11:G12"/>
+    <mergeCell ref="G13:I14"/>
+    <mergeCell ref="L13:N14"/>
+    <mergeCell ref="O13:O14"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="G15:G16"/>
+    <mergeCell ref="H15:H16"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="L15:L16"/>
+    <mergeCell ref="M15:N16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="G17:G18"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="M17:N18"/>
+    <mergeCell ref="H17:I18"/>
+    <mergeCell ref="K17:K18"/>
+    <mergeCell ref="L17:L18"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="H19:H20"/>
+    <mergeCell ref="I19:I20"/>
+    <mergeCell ref="D19:E20"/>
+    <mergeCell ref="K19:L20"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="M19:M20"/>
+    <mergeCell ref="N19:N20"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="D21:F22"/>
+    <mergeCell ref="J21:L22"/>
+    <mergeCell ref="M21:M22"/>
+    <mergeCell ref="N21:N22"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="G21:G22"/>
+    <mergeCell ref="H21:H22"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="E23:F24"/>
+    <mergeCell ref="N23:O24"/>
+    <mergeCell ref="G23:I24"/>
+    <mergeCell ref="L23:M24"/>
+    <mergeCell ref="K23:K24"/>
     <mergeCell ref="B25:B26"/>
     <mergeCell ref="D25:D26"/>
     <mergeCell ref="E25:E26"/>
@@ -5941,103 +6024,20 @@
     <mergeCell ref="H27:J28"/>
     <mergeCell ref="L27:L28"/>
     <mergeCell ref="M27:M28"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="D21:F22"/>
-    <mergeCell ref="J21:L22"/>
-    <mergeCell ref="M21:M22"/>
-    <mergeCell ref="N21:N22"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="D23:D24"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="G21:G22"/>
-    <mergeCell ref="H21:H22"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="E23:F24"/>
-    <mergeCell ref="N23:O24"/>
-    <mergeCell ref="G23:I24"/>
-    <mergeCell ref="L23:M24"/>
-    <mergeCell ref="K23:K24"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="H19:H20"/>
-    <mergeCell ref="I19:I20"/>
-    <mergeCell ref="D19:E20"/>
-    <mergeCell ref="K19:L20"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="M19:M20"/>
-    <mergeCell ref="N19:N20"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="G17:G18"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="M17:N18"/>
-    <mergeCell ref="H17:I18"/>
-    <mergeCell ref="K17:K18"/>
-    <mergeCell ref="L17:L18"/>
-    <mergeCell ref="O13:O14"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="G15:G16"/>
-    <mergeCell ref="H15:H16"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="L15:L16"/>
-    <mergeCell ref="M15:N16"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="K11:L12"/>
-    <mergeCell ref="N11:N12"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="J13:J14"/>
-    <mergeCell ref="K13:K14"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="M11:M12"/>
-    <mergeCell ref="E13:F14"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="I7:I8"/>
-    <mergeCell ref="D7:E8"/>
-    <mergeCell ref="G7:H8"/>
-    <mergeCell ref="L7:L8"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="K9:K10"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="L3:L4"/>
-    <mergeCell ref="M3:M4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="G3:G4"/>
-    <mergeCell ref="G5:H6"/>
-    <mergeCell ref="E5:F6"/>
-    <mergeCell ref="L5:L6"/>
-    <mergeCell ref="H3:J4"/>
-    <mergeCell ref="I5:K6"/>
-    <mergeCell ref="J7:K8"/>
-    <mergeCell ref="H9:J10"/>
-    <mergeCell ref="D9:E10"/>
-    <mergeCell ref="E11:G12"/>
-    <mergeCell ref="G13:I14"/>
-    <mergeCell ref="L13:N14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="N3:N4"/>
-    <mergeCell ref="M9:M10"/>
-    <mergeCell ref="N9:N10"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="I29:I30"/>
+    <mergeCell ref="J29:K30"/>
+    <mergeCell ref="F29:H30"/>
+    <mergeCell ref="L29:M30"/>
+    <mergeCell ref="N29:N30"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="G31:G32"/>
+    <mergeCell ref="H31:H32"/>
+    <mergeCell ref="I31:J32"/>
+    <mergeCell ref="N31:O32"/>
+    <mergeCell ref="K31:M32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="51" orientation="portrait" r:id="rId1"/>

</xml_diff>